<commit_message>
Repli WFS Géoplateforme pour Natura 2000 / ZNIEFF au clic ; couleur APB alignée sur les tuiles
- interrogerZonesProtegees : si l'API Carto échoue, repli sur le WFS (patrinat_*) ; si elle répond vide, repli sur les seules ZNIEFF marines
- Légende APB : couleur orange #ff8000 relevée sur les tuiles, note retirée
- Doc v1.9, tests (5sexies) et tableau de données à jour

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KC86j7E96GWSStyjvCXMe9
</commit_message>
<xml_diff>
--- a/data/donnees_carte_amidomar.xlsx
+++ b/data/donnees_carte_amidomar.xlsx
@@ -866,7 +866,8 @@
       <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Corrigé dans index.html le 21/09/2026 (endpoints natura-habitat et natura-oiseaux, champ sitename, délai porté à 8 s) et testé en réel sur 5 points (Port-Cros, Lavezzi, golfe du Morbihan, Beauduc, large de Quiberon). Non testé sur Brest. Le nom de site est bien identifié, mais les zones Natura 2000 restent affichées en image (voir lignes d'affichage).</t>
+          <t>Corrigé dans index.html le 21/09/2026 (endpoints natura-habitat et natura-oiseaux, champ sitename, délai porté à 8 s) et testé en réel sur 5 points (Port-Cros, Lavezzi, golfe du Morbihan, Beauduc, large de Quiberon). Non testé sur Brest. Le nom de site est bien identifié, mais les zones Natura 2000 restent affichées en image (voir lignes d'affichage).
+Repli branché le 21/09/2026 (v1.9) : si l'API Carto échoue, la carte interroge le WFS de la Géoplateforme (patrinat_sic, patrinat_zps). Test réel : l'API Carto a dépassé 8 s sur 2 requêtes Natura 2000 à Port-Cros, le repli a rendu « Rade d'Hyères » et « Iles d'Hyères ».</t>
         </is>
       </c>
     </row>
@@ -889,14 +890,13 @@
       <c r="D14" s="3" t="inlineStr"/>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>Ce qui ne va pas : le clic fonctionne, mais rien n'est renvoyé en mer sur les points testés.
-Ce qu'il faut : une source de clic pour les ZNIEFF marines.</t>
+          <t>Ce qui ne va pas : l'API Carto ne renvoie rien en mer pour les ZNIEFF. Un repli sur le WFS de la Géoplateforme (couches marines znieff1_mer et znieff2_mer) est branché depuis le 21/09/2026 ; il n'est confirmé que sur un point marin (Île Riou), pas sur la carte publiée.
+Ce qu'il faut : tester sur d'autres ZNIEFF marines connues une fois la version en ligne.</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>Tester le WFS de la Géoplateforme (patrinat_znieff1 et patrinat_znieff2) sur un point en mer, ou charger le jeu INPN complet (terrestre et marin) : https://www.data.gouv.fr/datasets/inpn-donnees-du-programme-znieff
-Piste testée le 21/09/2026 : le WFS de la Géoplateforme (couches patrinat_znieff1_mer et patrinat_znieff2_mer, filtre INTERSECTS sur le point cliqué) répond en mer ; voir les lignes d'affichage. Non branché dans la carte.</t>
+          <t>Repli WFS (v1.9) : patrinat_znieff1_mer et patrinat_znieff2_mer, filtre INTERSECTS sur le point cliqué. Test réel du 21/09/2026 : Île Riou → « ILE RIOU, ILOTS CONGLUÉ ET IMPÉRIAUX » (l'API Carto avait dépassé 8 s). Alternative : charger le jeu INPN complet : https://www.data.gouv.fr/datasets/inpn-donnees-du-programme-znieff</t>
         </is>
       </c>
     </row>
@@ -1138,7 +1138,7 @@
       <c r="D22" s="3" t="inlineStr"/>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>Ce qui ne va pas : la zone s'affiche comme une image, sans identification au clic. Le nom Patrinat_APB et les tuiles sont confirmés (test du 21/09/2026 : tuiles reçues sur 6 des 7 sites essayés, aucune à Hyères sur la tuile testée) ; l'affichage dans la carte elle-même n'a pas été vérifié à l'œil.
+          <t>Ce qui ne va pas : la zone s'affiche comme une image, sans identification au clic. Le nom Patrinat_APB et les tuiles sont confirmés (test du 21/09/2026 : tuiles reçues sur 6 des 7 sites essayés, aucune à Hyères sur la tuile testée) ; les APB s'affichent en orange vif (255, 128, 0), en fins contours et petits aplats, peu visibles quand on est dézoomé, et de couleur proche de celle des aires marines protégées ; des polygones orange sont visibles au Morbihan (zoom 11) sur la carte publiée, très probablement les APB (non confirmé en masquant la couche).
 Ce qu'il faut : ouvrir la carte publiée et vérifier le rendu, puis chercher les contours en données.</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Carte v2.4 à v2.6 : libellés, modale d'évitage concise, colonne d'eau estimée
- v2.4 : libellés (écosystèmes marins, AOT de mouillage existantes, message
  Natura 2000 avec étude d'incidence) ; couche Natura 2000 oiseaux cochée
  par défaut
- v2.5 : formulaire et résultat du rayon d'évitage dans la modale centrale ;
  bloc environnement réduit à une ligne avec « Détails » quand un mouillage
  est proche ; suppression du bloc « Calcul rayon d'évitage » à droite
- v2.6 : colonne d'eau à marée haute pré-remplie (profondeur EMODnet +
  marée haute de vives-eaux du port de référence le plus proche, table
  data/ram-ports.json issue des RAM du Shom), modifiable
- Documentation, tests et tableau des données mis à jour

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BiwtttreAhE9oSHnDpHopw
</commit_message>
<xml_diff>
--- a/data/donnees_carte_amidomar.xlsx
+++ b/data/donnees_carte_amidomar.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1029,59 +1029,89 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>Bathymétrie</t>
+          <t>Profondeur au point (colonne d'eau à marée haute)</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Aucune</t>
+          <t>EMODnet Bathymetry, API depth_sample (grille européenne intégrant les levés du Shom)</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>JSON (REST), maille d'environ 115 m</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr"/>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>Ce qui ne va pas : aucune profondeur disponible, l'usager la saisit à la main, donc le rayon d'évitage n'est qu'indicatif.
-Ce qu'il faut : un fichier de profondeurs marines lisible au point cliqué.</t>
+          <t>Ce qui ne va pas : branché en v2.6 (25/09/2026) et testé sur l'API réelle, mais le clic complet sur la carte publiée avec l'API réelle reste à vérifier ; la maille d'environ 115 m donne un fond moyen, peu fidèle près des roches et des chenaux.
+Ce qu'il faut : un test en conditions réelles sur la carte publiée, puis, si besoin, une bathymétrie plus fine sur les zones pilotes (MNT côtiers du Shom à 5-20 m).</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>MNT de façade du Shom (projet Homonim), gratuits en licence ouverte, résolution 0,001° soit environ 111 m, en formats ASC, GLZ, BAG, GRD, à télécharger par zone. Ce sont des grilles à convertir avant usage sur la carte, et 111 m est grossier près du rivage (mon évaluation).
-Atlantique, Manche, mer du Nord : https://diffusion.shom.fr/donnees/bathymerie/mnt-facade-atl-homonim.html
-Golfe du Lion - Côte d'Azur : https://diffusion.shom.fr/mnt-facade-gdl-ca-homonim.html
-Corse : https://diffusion.shom.fr/mnt-facade-atl-homonim_1.html</t>
+          <t>API testée le 25/09/2026 depuis le site publié : CORS accepté, 60 à 370 ms ; Quiberon −12,35 m, Brest −23,6 m, Saint-Malo −1,86 m. https://rest.emodnet-bathymetry.eu/depth_sample?geom=POINT(-2.970485 47.510572)
+Écartés : WMS « MNT » du Shom non interrogeable au point (LayerNotQueryable), export image/x-bil incohérent (tests du 25/09/2026).
+Plus fin (non testé) : MNT côtiers du Shom à 5-20 m (Morbihan, Pertuis, Arcachon, Île de Ré, Gironde…) visibles dans le WMS INSPIRE, à télécharger et convertir : https://diffusion.shom.fr/donnees/bathymerie/mnt-bathymetriques.html
+MNT de façade Homonim (111 m, Licence Ouverte) : https://www.data.gouv.fr/datasets/mnt-bathymetrique-de-facade-atlantique-projet-homonim-1</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>Hauteur de marée haute (colonne d'eau à marée haute)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>data/ram-ports.json, extrait du Shom, Références Altimétriques Maritimes (WFS RAM_BDD_WLD_WGS84G_WFS:ram_3857)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>JSON, 214 ports (métropole)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n"/>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Ce qui ne va pas : valeur fixe par port (vives-eaux moyennes, coefficient 95), pas la marée du jour ; port choisi à vol d'oiseau, parfois de l'autre côté d'une pointe ; 15 ports sans valeurs exploitables écartés ; extraction du 25/09/2026 à rafraîchir si le Shom publie une nouvelle édition.
+Ce qu'il faut : garder la table à jour ; pour la marée du jour, un abonnement aux API de prédiction du Shom (payant) avec un petit serveur intermédiaire.</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>Source ouverte (Licence Ouverte, citer « Shom, 2025 ») : https://www.data.gouv.fr/datasets/references-altimetriques-maritimes — WFS interrogé le 25/09/2026 (446 sites, 229 en métropole, sommes de contrôle notées dans TESTS_FONCTIONNELS.md §5/9quinquies).
+API marée du Shom (payantes, clé) : https://diffusion.shom.fr/api-shom.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
           <t>Vent, courant, nature du fond</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Aucune</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Ce qui ne va pas : le calcul du rayon d'évitage ignore le vent, le courant et le type de fond, qui changent la zone réellement balayée par le bateau.
 Ce qu'il faut : ces trois données.</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>Nature du fond : Natures de fond au 1/50 000 (Shom), 47 cartes, shapefile et GML, WMS/WMTS/WFS, gratuit, version 2025 : https://diffusion.shom.fr/donnees/sedimentologie/natures-de-fond.html
 Courants : la page Shom des courants de marée 2D était inaccessible au test, et l'API Shom ne liste ni courants ni vent (marées payantes) : https://diffusion.shom.fr/services-numeriques/api-shom.html
@@ -1090,142 +1120,142 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Réserves naturelles nationales</t>
         </is>
       </c>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>Patrinat_RNN (Géoplateforme)</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>Non testé</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="3" t="inlineStr">
         <is>
           <t>Ce qui ne va pas : la couche existe mais n'est pas sur la carte, alors que la note la donne « en service ».
 Ce qu'il faut : l'ajouter et la tester.</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>Couche patrinat_rnn confirmée dans le document de capacités WFS de la Géoplateforme (21/09/2026) : https://data.geopf.fr/wfs?REQUEST=GetCapabilities&amp;SERVICE=WFS&amp;VERSION=2.0.0</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>Arrêtés de protection de biotope (APB)</t>
         </is>
       </c>
-      <c r="B22" s="2" t="inlineStr">
+      <c r="B23" s="2" t="inlineStr">
         <is>
           <t>IGN / INPN, Patrinat_APB</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C23" s="2" t="inlineStr">
         <is>
           <t>WMTS, tuiles PNG raster</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>données fonctionnelles</t>
         </is>
       </c>
-      <c r="E22" s="2" t="n"/>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Affichage : couche patrinat_apb confirmée en WFS et en WMTS le 21/09/2026 ; polygones vus au Morbihan (zoom 11), couleur de légende orange alignée sur les tuiles.
 Au clic (v2.0, 22/09/2026) : couche patrinat_apb:apb, champ nom_site, filtre INTERSECTS. Testé en direct sur l'APB « Ile Dumet et ses abords » (centre du polygone, pas un sommet) : nom renvoyé en ~480 ms. Traité comme une interdiction bloquante, prioritaire sur Natura 2000/ZNIEFF (popup rouge, pas de coordonnées), vérifiée avant tout affichage (délai 4 s, défaut non bloquant). Reste à tester : un clic réel dans un APB sur la carte publiée.</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t>Autres zonages (Ramsar, RNR, Conservatoire du littoral)</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B24" s="3" t="inlineStr">
         <is>
           <t>Patrinat_RAMSAR, Patrinat_RNR, CONSERVATOIRE_LITTORAL.PERIMETRES</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C24" s="3" t="inlineStr">
         <is>
           <t>Non testé</t>
         </is>
       </c>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr">
         <is>
           <t>Ce qui ne va pas : couches existantes mais absentes de la carte.
 Ce qu'il faut : décider si le besoin métier justifie de les ajouter, puis vérifier le rendu.</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F24" s="3" t="inlineStr">
         <is>
           <t>WFS Géoplateforme : patrinat_ramsar et CONSERVATOIRE_LITTORAL.PERIMETRES sont listées ; patrinat_rnr y figure aussi (noms confirmés le 21/09/2026 ; requêtes de données non testées) : https://data.geopf.fr/wfs?REQUEST=GetCapabilities&amp;SERVICE=WFS&amp;VERSION=2.0.0
 Espaces protégés du Conservatoire du littoral (titre repéré, non ouvert) : https://www.data.gouv.fr/datasets/site-des-espaces-proteges-du-conservatoire-du-littoral</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Zones de baignade et zones réglementaires</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Aucune</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D24" s="3" t="n"/>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="inlineStr">
         <is>
           <t>Ce qui ne va pas : ligne « à venir » dans la légende, grisée et non sélectionnable. Aucune source n'est identifiée pour représenter ces zones ni les reconnaître au clic.
 Ce qu'il faut : identifier une source pour chacune des deux.</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F25" s="3" t="inlineStr">
         <is>
           <t>Aucune source confirmée. Pistes non vérifiées : données de baignade publiées par les communes ou les ARS, arrêtés préfectoraux à demander aux DDTM/DM.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="5" t="n"/>
-    </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr">
-        <is>
-          <t>Légende : vert = données fonctionnelles ; jaune = données simulées ; sans couleur = à compléter.</t>
-        </is>
-      </c>
+      <c r="A26" s="5" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Méthode (21/09/2026) : les fiches de jeux de données ont été ouvertes et lues ; les services WMS/WFS et les fichiers n'ont pas été interrogés ni téléchargés. « Titre repéré, non ouvert » = trouvé par recherche seulement.</t>
+          <t>Légende : vert = données fonctionnelles ; jaune = données simulées ; sans couleur = à compléter.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Méthode (21/09/2026) : les fiches de jeux de données ont été ouvertes et lues ; les services WMS/WFS et les fichiers n'ont pas été interrogés ni téléchargés. « Titre repéré, non ouvert » = trouvé par recherche seulement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Le document de capacités WFS et WMTS de la Géoplateforme a été interrogé dans un navigateur le 21/09/2026 : les noms de couches patrinat_* cités ici y figurent. Aucune requête de données (GetFeature) n'a encore été testée.</t>
         </is>
@@ -1242,7 +1272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1831,7 +1861,7 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Bathymétrie</t>
+          <t>Profondeur au point (colonne d'eau à marée haute)</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
@@ -1848,7 +1878,7 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Bathymétrie</t>
+          <t>Profondeur au point (colonne d'eau à marée haute)</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
@@ -1865,7 +1895,7 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Bathymétrie</t>
+          <t>Profondeur au point (colonne d'eau à marée haute)</t>
         </is>
       </c>
       <c r="B37" s="8" t="inlineStr">
@@ -1995,6 +2025,91 @@
       <c r="C44" s="7" t="inlineStr">
         <is>
           <t>Repéré en recherche, non ouvert</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Profondeur au point (colonne d'eau à marée haute)</t>
+        </is>
+      </c>
+      <c r="B45" s="8" t="inlineStr">
+        <is>
+          <t>https://www.data.gouv.fr/datasets/mnt-bathymetrique-de-facade-atlantique-projet-homonim-1</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>Page ouverte le 25/09/2026 (licence, résolution et ressources lues ; WMS non interrogé)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Profondeur au point (colonne d'eau à marée haute)</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t>https://diffusion.shom.fr/api-shom.html</t>
+        </is>
+      </c>
+      <c r="C46" s="7" t="inlineStr">
+        <is>
+          <t>Page ouverte le 25/09/2026 (API marée payantes avec clé)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Profondeur au point (colonne d'eau à marée haute)</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>https://services.data.shom.fr/support/en/services/spm</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>Page ouverte le 25/09/2026 (SPM/SAPM : clé d'abonnement obligatoire)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Profondeur au point (colonne d'eau à marée haute)</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>https://rest.emodnet-bathymetry.eu/depth_sample?geom=POINT(-2.970485 47.510572)</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>API interrogée le 25/09/2026 depuis le site publié (réponse JSON, CORS OK)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Hauteur de marée haute (colonne d'eau à marée haute)</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>https://www.data.gouv.fr/datasets/references-altimetriques-maritimes</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>Fiche lue le 25/09/2026 (licence, ressources) ; WFS du Shom interrogé le même jour</t>
         </is>
       </c>
     </row>
@@ -2043,6 +2158,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId42"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId48"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Carte v2.10 : vraies données ZMEL branchées sur la carte
- data/zmel.geojson remplacé par les 647 vraies ZMEL (Cerema/CACEM,
  France entière et Antilles) au lieu de l'unique zone fictive
  précédente (Nicolas a signalé qu'aucune ZMEL ne s'affichait sur la
  carte). data/zmel-reel.geojson conservé comme copie de référence.
- Note de la couche « ZMEL » (légende) et note de bas de modale mises à
  jour : ne mentionnent plus de données fictives, statut passé de
  `local` à `verifie`.
- Jeu de secours hors-ligne (double-clic sur index.html) remplacé par
  3 vraies ZMEL au lieu de l'exemple fictif « ZMEL à remplacer ».
- Documentation fonctionnelle, tests fonctionnels et classeur de suivi
  des données synchronisés ; testé en HTTP réel (pas file://) pour
  confirmer que le fetch charge bien les 647 features et pas le
  fallback de secours.

Non vérifié sur la version publiée (à faire après push).
</commit_message>
<xml_diff>
--- a/data/donnees_carte_amidomar.xlsx
+++ b/data/donnees_carte_amidomar.xlsx
@@ -901,42 +901,37 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="2" t="inlineStr">
         <is>
           <t>ZMEL</t>
         </is>
       </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>data/zmel.geojson</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>GeoJSON, 1 polygone fictif</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr"/>
-      <c r="E15" s="4" t="inlineStr">
-        <is>
-          <t>données simulées</t>
-        </is>
-      </c>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>Méditerranée (Corse, Languedoc-Roussillon, PACA) : jeu DIRM Méditerranée, shapefile, WMS/WFS, Licence Ouverte 2.0, publié en 2021. Attention : c'est une interprétation des textes, pas la réglementation officielle. Il peut aussi combler le jeu du Var signalé en panne. https://catalogue.sigena.fr/geonetwork/srv/api/records/fr-120066022-jdd-86ec0654-0c2c-4e76-a9a0-abb36d978d34
-Charente-Maritime (DDTM 17) : shapefile, WMS/WFS, mis à jour en 2024 : https://www.data.gouv.fr/datasets/zones-de-mouillages-et-dequipements-legers-zmel-en-charente-maritime
-Finistère (DDTM 29, jeu archivé, donnée d'avril 2025) : https://www.data.gouv.fr/datasets/mouillages-groupes-du-finistere-1/
-Morbihan (titre repéré, non ouvert) : https://www.data.gouv.fr/datasets/zones-de-mouillage-et-dequipements-legers-zmel-departement-du-morbihan-1
-Vue nationale : 260 ZMEL dans 209 communes sur GéoLittoral, sans téléchargement annoncé ; demande possible à geolittoral@cerema.fr : https://www.geolittoral.developpement-durable.gouv.fr/zones-de-mouillage-et-d-equipements-legers-a1757.html?lang=fr
-25/09/2026 : Nicolas a fourni un shapefile Cerema/CACEM (647 ZMEL, France entière) — converti dans data/zmel-reel.geojson (voir ligne ci-dessous), mais pas encore branché ici.</t>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>data/zmel.geojson — shapefile Cerema/CACEM fourni par Nicolas (ZMEL_18_09_2026), converti et branché</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>GeoJSON, 647 polygones/multipolygones, France entière + Antilles</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>données fonctionnelles</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Branché le 25/09/2026 (v2.10), remplace l'ancien fichier fictif. Reste à améliorer : nb_postes_ est un total agrégé en texte (pas de détail par catégorie de navire affiché) ; aucun contact e-mail dans la source (voir ligne ci-dessous pour le détail de la conversion et la tentative infructueuse de récupération de contacts via Légicem). Champs redev_an_z/redev_an_p (redevance) présents dans la donnée mais volontairement pas affichés au public.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>ZMEL (données réelles converties, non branchées)</t>
+          <t>ZMEL — source de la conversion (shapefile d'origine)</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
@@ -952,7 +947,7 @@
       <c r="D16" s="4" t="n"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>Converti et vérifié géométriquement (bbox plausible, 0 entité perdue) le 25/09/2026, mais PAS ENCORE branché sur la carte (data/zmel.geojson, fictif, reste la source active). Schéma d'attributs différent de celui attendu par modaleZmel() : nb_postes_ est un total agrégé en texte (pas de nombre par navire simple), pas de champ e-mail/contact. Lien url_v2 (fiches Légicem) injoignable depuis l'extérieur : domaine legicem.metier.e2.rie.gouv.fr sur le RIE (réseau interministériel de l'État), échec de connexion confirmé le 25/09/2026 — inutilisable pour récupérer un contact, y compris pour le public. Champ redev_an_z/redev_an_p (redevance) présent mais volontairement pas prévu à l'affichage public (sensible).</t>
+          <t>Converti et vérifié géométriquement (bbox plausible, 0 entité perdue) le 25/09/2026, puis branché sur la carte le même jour (v2.10) : data/zmel.geojson est désormais une copie conforme de ce fichier. Schéma d'attributs différent de celui attendu par modaleZmel() : nb_postes_ est un total agrégé en texte (pas de nombre par navire simple), pas de champ e-mail/contact. Lien url_v2 (fiches Légicem) injoignable depuis l'extérieur : domaine legicem.metier.e2.rie.gouv.fr sur le RIE (réseau interministériel de l'État), échec de connexion confirmé le 25/09/2026 — inutilisable pour récupérer un contact, y compris pour le public. Champ redev_an_z/redev_an_p (redevance) présent mais volontairement pas prévu à l'affichage public (sensible).</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">

</xml_diff>

<commit_message>
v2.22 : rattachement DDTM au clic et dégagement du point sous le popup
</commit_message>
<xml_diff>
--- a/data/donnees_carte_amidomar.xlsx
+++ b/data/donnees_carte_amidomar.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1365,25 +1365,81 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="5" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Légende : vert = données fonctionnelles ; jaune = données simulées ; sans couleur = à compléter.</t>
+    <row r="29" ht="150" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Rattachement départemental au clic (quelle DDTM ?)</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>SHOM-IGN, LIMTM 2021, services INSPIRE — attribut numdep de la couche limite_terre_mer_france_metropolitaine_polygones</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>WFS 2.0.0, GeoJSON, filtre DWITHIN à rayons progressifs (1, 2, 5, 10 km)</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>données fonctionnelles</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr"/>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Branché le 14/10/2026 (v2.22), sans nouvelle source : la couche était déjà interrogée depuis la v2.14 et renvoyait déjà numdep. Calibrage vérifié en réel le 14/10/2026 sur 6 points (rade de Brest 29, golfe du Morbihan 56, rade de Toulon 83, Les Sept-Îles 22, baie de Saint-Brieuc 22) : réponse univoque à chaque fois. LIMITE À CONNAÎTRE : la couche porte des surfaces TERRESTRES, le département est donc celui de la côte la plus proche, jamais celui du point cliqué — c'est une inférence, et aucune limite départementale ne s'étend en mer dans ce jeu. Piste pour lever cette limite : demander au Shom (Eric Le Guen, équipe zones et limites maritimes) s'il existe un référentiel de limites administratives EN MER diffusable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="150" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Messages d'orientation par DDTM (règles locales)</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>data/ddtm-messages.json — rédigé par l'équipe, en attendant l'interface instructeur Grist</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>JSON, texte brut échappé à l'affichage, 2 fiches (22 et 83)</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr"/>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Ce qui ne va pas : les zones dédiées du Var (83) ne sont pas renseignées — 4 entrées « À COMPLÉTER ». Le drapeau brouillon est posé et la carte affiche « information provisoire », mais ces zones doivent être obtenues auprès de la DDTM 83 avant toute communication publique. Le 29 et le 56 n'ont pas de message, ce qui est normal à ce jour.</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Fichier PROVISOIRE par conception : il sera régénéré depuis la table DDTM de Grist quand l'interface instructeur permettra aux agents de gérer leurs bandeaux par périmètre en autonomie. Ses noms de champs sont déjà ceux prévus pour cette table (ddtm, message_titre, message_consequence, message_detail, liste, lien, libelle_lien), pour que le basculement soit un script d'export et non une réécriture de la carte. Secours hors ligne volontairement vide.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>Méthode (21/09/2026) : les fiches de jeux de données ont été ouvertes et lues ; les services WMS/WFS et les fichiers n'ont pas été interrogés ni téléchargés. « Titre repéré, non ouvert » = trouvé par recherche seulement.</t>
-        </is>
-      </c>
+      <c r="A31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Légende : vert = données fonctionnelles ; jaune = données simulées ; sans couleur = à compléter.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Méthode (21/09/2026) : les fiches de jeux de données ont été ouvertes et lues ; les services WMS/WFS et les fichiers n'ont pas été interrogés ni téléchargés. « Titre repéré, non ouvert » = trouvé par recherche seulement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Le document de capacités WFS et WMTS de la Géoplateforme a été interrogé dans un navigateur le 21/09/2026 : les noms de couches patrinat_* cités ici y figurent. Aucune requête de données (GetFeature) n'a encore été testée.</t>
         </is>

</xml_diff>

<commit_message>
v2.23 : cadre complet sur la règle locale, zones AOT du Var en GeoJSON, cliquables et affichées
</commit_message>
<xml_diff>
--- a/data/donnees_carte_amidomar.xlsx
+++ b/data/donnees_carte_amidomar.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1393,7 +1393,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="150" customHeight="1">
+    <row r="30" ht="190" customHeight="1">
       <c r="A30" s="11" t="inlineStr">
         <is>
           <t>Messages d'orientation par DDTM (règles locales)</t>
@@ -1406,40 +1406,68 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>JSON, texte brut échappé à l'affichage, 2 fiches (22 et 83)</t>
+          <t>JSON, texte brut échappé à l'affichage, 2 fiches (22 et 83), 5 zones listées pour le 83</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr"/>
       <c r="E30" s="11" t="inlineStr">
         <is>
-          <t>Ce qui ne va pas : les zones dédiées du Var (83) ne sont pas renseignées — 4 entrées « À COMPLÉTER ». Le drapeau brouillon est posé et la carte affiche « information provisoire », mais ces zones doivent être obtenues auprès de la DDTM 83 avant toute communication publique. Le 29 et le 56 n'ont pas de message, ce qui est normal à ce jour.</t>
+          <t>Ce qui ne va pas : la liste des zones du Var est partielle. Les 5 zones reçues de la DDTM 83 (cartes PDF n°41 Les Canebiers et n°42 La Bouillabaisse, octobre 2022) sont toutes sur la commune de Saint-Tropez, alors que la DDTM 83 couvre toute la façade varoise. Le texte de la carte l'annonce et le drapeau brouillon reste posé, mais il faut obtenir les zones des autres communes (Hyères, Giens, Porquerolles, Cavalaire, Le Lavandou, Bandol...). Le 29 et le 56 n'ont pas de message, ce qui est normal à ce jour.</t>
         </is>
       </c>
       <c r="F30" s="11" t="inlineStr">
         <is>
-          <t>Fichier PROVISOIRE par conception : il sera régénéré depuis la table DDTM de Grist quand l'interface instructeur permettra aux agents de gérer leurs bandeaux par périmètre en autonomie. Ses noms de champs sont déjà ceux prévus pour cette table (ddtm, message_titre, message_consequence, message_detail, liste, lien, libelle_lien), pour que le basculement soit un script d'export et non une réécriture de la carte. Secours hors ligne volontairement vide.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="n"/>
+          <t>Fichier PROVISOIRE par conception : il sera régénéré depuis la table DDTM de Grist quand l'interface instructeur permettra aux agents de gérer leurs bandeaux par périmètre en autonomie. Ses noms de champs sont déjà ceux prévus pour cette table. PISTE NON ENGAGÉE : les deux cartes PDF donnent les 4 sommets GPS de chaque zone (degrés-minutes décimales). Les convertir en polygones GeoJSON permettrait de répondre directement à la question de l'usager (« mon emplacement est-il dans une zone autorisée ? ») au lieu de lui faire lire une liste de noms, et d'afficher les zones sur la carte comme les ZMEL. Secours hors ligne volontairement vide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="190" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Zones de mouillage autorisées (AOT)</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>data/zones-aot.geojson — relevé manuel sur les cartes PDF n°41 et n°42 de la DDTM du Var / SML-BLO, octobre 2022</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>GeoJSON, 5 polygones (4 sommets chacun), propriétés : ddtm, commune, lieu, zone, capacité, exposition, profondeur</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr"/>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Ce qui ne va pas : couverture très partielle (5 zones, commune de Saint-Tropez uniquement) et saisie non validée. Les coordonnées ont été lues à l'oeil sur des PDF : une erreur déplacerait une limite réglementaire. Il faut (1) faire confirmer les sommets par la DDTM 83, (2) vérifier que les cartes d'octobre 2022 sont toujours en vigueur, (3) obtenir les zones des autres communes varoises.</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Contrôle de cohérence déjà fait : surface du polygone divisée par la capacité annoncée = 937, 1016, 863, 914 et 1065 m2 par mouillage sur les cinq zones, soit environ 18 m de rayon d'évitage. Cette convergence écarte la faute de frappe mais ne vaut pas validation. Le fichier sert deux fois : couche cartographique (id zones_aot) et liste cliquable du message DDTM, reliées par la propriété ddtm. Demander à la DDTM 83 un export SIG plutôt que des PDF pour les prochaines communes.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>Légende : vert = données fonctionnelles ; jaune = données simulées ; sans couleur = à compléter.</t>
-        </is>
-      </c>
+      <c r="A32" s="5" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Méthode (21/09/2026) : les fiches de jeux de données ont été ouvertes et lues ; les services WMS/WFS et les fichiers n'ont pas été interrogés ni téléchargés. « Titre repéré, non ouvert » = trouvé par recherche seulement.</t>
+          <t>Légende : vert = données fonctionnelles ; jaune = données simulées ; sans couleur = à compléter.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>Méthode (21/09/2026) : les fiches de jeux de données ont été ouvertes et lues ; les services WMS/WFS et les fichiers n'ont pas été interrogés ni téléchargés. « Titre repéré, non ouvert » = trouvé par recherche seulement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Le document de capacités WFS et WMTS de la Géoplateforme a été interrogé dans un navigateur le 21/09/2026 : les noms de couches patrinat_* cités ici y figurent. Aucune requête de données (GetFeature) n'a encore été testée.</t>
         </is>

</xml_diff>

<commit_message>
v2.24 : règle locale au vert dans une zone autorisée, et correction du faux positif « fond de carte indisponible »
</commit_message>
<xml_diff>
--- a/data/donnees_carte_amidomar.xlsx
+++ b/data/donnees_carte_amidomar.xlsx
@@ -510,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F35"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -1406,7 +1406,7 @@
       </c>
       <c r="C30" s="11" t="inlineStr">
         <is>
-          <t>JSON, texte brut échappé à l'affichage, 2 fiches (22 et 83), 5 zones listées pour le 83</t>
+          <t>JSON, texte brut échappé à l'affichage, 2 fiches (22 et 83). Le 83 porte deux jeux de textes : l'état par défaut et l'état « emplacement dans une zone autorisée » (champs *_zone, v2.24)</t>
         </is>
       </c>
       <c r="D30" s="11" t="inlineStr"/>
@@ -1421,53 +1421,25 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="190" customHeight="1">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>Zones de mouillage autorisées (AOT)</t>
-        </is>
-      </c>
-      <c r="B31" s="11" t="inlineStr">
-        <is>
-          <t>data/zones-aot.geojson — relevé manuel sur les cartes PDF n°41 et n°42 de la DDTM du Var / SML-BLO, octobre 2022</t>
-        </is>
-      </c>
-      <c r="C31" s="11" t="inlineStr">
-        <is>
-          <t>GeoJSON, 5 polygones (4 sommets chacun), propriétés : ddtm, commune, lieu, zone, capacité, exposition, profondeur</t>
-        </is>
-      </c>
-      <c r="D31" s="11" t="inlineStr"/>
-      <c r="E31" s="11" t="inlineStr">
-        <is>
-          <t>Ce qui ne va pas : couverture très partielle (5 zones, commune de Saint-Tropez uniquement) et saisie non validée. Les coordonnées ont été lues à l'oeil sur des PDF : une erreur déplacerait une limite réglementaire. Il faut (1) faire confirmer les sommets par la DDTM 83, (2) vérifier que les cartes d'octobre 2022 sont toujours en vigueur, (3) obtenir les zones des autres communes varoises.</t>
-        </is>
-      </c>
-      <c r="F31" s="11" t="inlineStr">
-        <is>
-          <t>Contrôle de cohérence déjà fait : surface du polygone divisée par la capacité annoncée = 937, 1016, 863, 914 et 1065 m2 par mouillage sur les cinq zones, soit environ 18 m de rayon d'évitage. Cette convergence écarte la faute de frappe mais ne vaut pas validation. Le fichier sert deux fois : couche cartographique (id zones_aot) et liste cliquable du message DDTM, reliées par la propriété ddtm. Demander à la DDTM 83 un export SIG plutôt que des PDF pour les prochaines communes.</t>
-        </is>
-      </c>
+    <row r="31">
+      <c r="A31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="5" t="n"/>
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>Légende : vert = données fonctionnelles ; jaune = données simulées ; sans couleur = à compléter.</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>Légende : vert = données fonctionnelles ; jaune = données simulées ; sans couleur = à compléter.</t>
+          <t>Méthode (21/09/2026) : les fiches de jeux de données ont été ouvertes et lues ; les services WMS/WFS et les fichiers n'ont pas été interrogés ni téléchargés. « Titre repéré, non ouvert » = trouvé par recherche seulement.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
-        <is>
-          <t>Méthode (21/09/2026) : les fiches de jeux de données ont été ouvertes et lues ; les services WMS/WFS et les fichiers n'ont pas été interrogés ni téléchargés. « Titre repéré, non ouvert » = trouvé par recherche seulement.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="5" t="inlineStr">
         <is>
           <t>Le document de capacités WFS et WMTS de la Géoplateforme a été interrogé dans un navigateur le 21/09/2026 : les noms de couches patrinat_* cités ici y figurent. Aucune requête de données (GetFeature) n'a encore été testée.</t>
         </is>

</xml_diff>